<commit_message>
Sync local workspace snapshot: v14 BPMN model, 36 Camunda forms, docs, workers, tools, diagrams, screenshots
</commit_message>
<xml_diff>
--- a/docs/GroupMj Sprint-1-Backlog.xlsx
+++ b/docs/GroupMj Sprint-1-Backlog.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17260"/>
+    <workbookView windowWidth="32740" windowHeight="16140"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="75">
   <si>
     <t>Sprint 1:  2026-09-15  →  2026-09-21</t>
   </si>
@@ -38,54 +38,40 @@
     <t>Deliver the core end-to-end path: referral intake → document check → consultant review → acceptance → new patient appointment → treatment request.</t>
   </si>
   <si>
-    <t>交付核心端到端路径：转诊接收 → 文件检查 → 顾问审核 → 接受 → 新患者预约 → 治疗请求。</t>
-  </si>
-  <si>
-    <t>Group
-组</t>
-  </si>
-  <si>
-    <t>Workpackage
-工作包</t>
-  </si>
-  <si>
-    <t>Item ID
-任务名</t>
-  </si>
-  <si>
-    <t>Content
-内容</t>
-  </si>
-  <si>
-    <t>First Owner
-第一负责人</t>
-  </si>
-  <si>
-    <t>Second Owner
-第二负责人</t>
-  </si>
-  <si>
-    <t>Story Points
-故事点</t>
-  </si>
-  <si>
-    <t>Deliverable / Due
-交付物 / 完成日</t>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Workpackage</t>
+  </si>
+  <si>
+    <t>Item ID</t>
+  </si>
+  <si>
+    <t>Content</t>
+  </si>
+  <si>
+    <t>First Owner</t>
+  </si>
+  <si>
+    <t>Second Owner</t>
+  </si>
+  <si>
+    <t>Story Points</t>
+  </si>
+  <si>
+    <t>Deliverable / Due</t>
   </si>
   <si>
     <t>G1-1</t>
   </si>
   <si>
-    <t xml:space="preserve">
-Project management
-项目管理</t>
+    <t>Project management</t>
   </si>
   <si>
     <t>Mj01, Mj03-Mj07</t>
   </si>
   <si>
-    <t>Project kickoff, backlog, SU1/SR1 records, retrospective
-项目启动、Backlog、SU1/SR1 记录、回顾</t>
+    <t>Project kickoff, backlog, SU1/SR1 records, retrospective</t>
   </si>
   <si>
     <t>T</t>
@@ -95,7 +81,6 @@
   </si>
   <si>
     <t>Charter, backlog workbook v1.0, SU1/SR1 logs, retrospective minutes
-团队章程、Backlog v1.0、SU1/SR1 记录、回顾记录
 due: Day 1 – Day 6-7</t>
   </si>
   <si>
@@ -105,35 +90,29 @@
     <t>Mj02</t>
   </si>
   <si>
-    <t>Scope boundary, stakeholder map, assumption list
-范围边界、干系人图、假设清单</t>
+    <t>Scope boundary, stakeholder map, assumption list</t>
   </si>
   <si>
     <t>D</t>
   </si>
   <si>
     <t>Scope section, stakeholder map, numbered assumptions
-范围章节、干系人图、编号假设清单
 due: Day 1-2</t>
   </si>
   <si>
     <t>G2-1</t>
   </si>
   <si>
-    <t xml:space="preserve">
-Requirements
-需求类</t>
+    <t>Requirements</t>
   </si>
   <si>
     <t>Mj11</t>
   </si>
   <si>
-    <t>Functional requirements list and traceability
-功能需求清单与追溯表</t>
+    <t>Functional requirements list and traceability</t>
   </si>
   <si>
     <t>FRS with traceability to backlog IDs
-FRS 及到待办编号的追溯表
 due: Day 1-2</t>
   </si>
   <si>
@@ -143,15 +122,13 @@
     <t>Mj13</t>
   </si>
   <si>
-    <t>Data and variable dictionary
-数据与变量字典</t>
+    <t>Data and variable dictionary</t>
   </si>
   <si>
     <t>L</t>
   </si>
   <si>
     <t>Data dictionary cross-checked against models
-数据字典，已与模型交叉核对
 due: Day 2</t>
   </si>
   <si>
@@ -161,32 +138,26 @@
     <t>Mj14</t>
   </si>
   <si>
-    <t>External service interface definitions
-外部服务接口定义</t>
+    <t>External service interface definitions</t>
   </si>
   <si>
     <t>Interface contracts for four simulated services
-四个模拟服务的接口契约
 due: Day 5</t>
   </si>
   <si>
     <t>G3-1</t>
   </si>
   <si>
-    <t xml:space="preserve">
-BPMNcore
-BPMN 核心</t>
+    <t>BPMNcore</t>
   </si>
   <si>
     <t>Mj15, Mj28</t>
   </si>
   <si>
-    <t>Multi-pool collaboration diagram and deployment configuration
-多池协作图与部署配置</t>
+    <t>Multi-pool collaboration diagram and deployment configuration</t>
   </si>
   <si>
     <t>Collaboration model + deployable configuration package
-协作模型 + 可部署配置包
 due: Day 3-4</t>
   </si>
   <si>
@@ -196,12 +167,10 @@
     <t>Mj16, Mj17</t>
   </si>
   <si>
-    <t>Referral intake and consultant clinical review
-转诊接收与顾问临床审核</t>
+    <t>Referral intake and consultant clinical review</t>
   </si>
   <si>
     <t>Referral process model, four review outcomes testable
-转诊流程模型，四种审核结果均可执行
 due: Day 3-4</t>
   </si>
   <si>
@@ -211,12 +180,10 @@
     <t>Mj18</t>
   </si>
   <si>
-    <t>New patient appointment booking and patient notification
-新患者预约与患者通知</t>
+    <t>New patient appointment booking and patient notification</t>
   </si>
   <si>
     <t>Appointment model incl. two-week telephone rule
-预约模型，含两周内电话联系规则
 due: Day 4-5</t>
   </si>
   <si>
@@ -226,12 +193,10 @@
     <t>Mj19</t>
   </si>
   <si>
-    <t>Informed consent and authorised treatment request
-知情同意与授权治疗申请</t>
+    <t>Informed consent and authorised treatment request</t>
   </si>
   <si>
     <t>Consent capture + clinician-only authorisation gate
-知情同意记录 + 仅临床可授权的拦截点
 due: Day 4-5</t>
   </si>
   <si>
@@ -241,12 +206,10 @@
     <t>Mj20</t>
   </si>
   <si>
-    <t>Treatment appointment coordination
-治疗预约协调</t>
+    <t>Treatment appointment coordination</t>
   </si>
   <si>
     <t>Treatment booking model incl. service-unavailable pending path
-治疗预约模型，含服务不可用待处理路径
 due: Day 5</t>
   </si>
   <si>
@@ -260,12 +223,10 @@
     <t>Mj29, Mj30, Mj34</t>
   </si>
   <si>
-    <t>Scheduling and communication workers, environment configuration
-调度与通信 Worker、环境配置</t>
+    <t>Scheduling and communication workers, environment configuration</t>
   </si>
   <si>
     <t>Two workers + secret and configuration templates
-两个 Worker + 密钥与配置模板
 due: Day 1-4</t>
   </si>
   <si>
@@ -279,37 +240,27 @@
     <t>Mj36-Mj39</t>
   </si>
   <si>
-    <t>Core Camunda forms
-核心 Camunda Forms</t>
+    <t>Core Camunda forms</t>
   </si>
   <si>
     <t>Four forms + variable binding table
-四张表单 + 变量绑定表
 due: Day 2-5</t>
   </si>
   <si>
     <t>G6-1</t>
   </si>
   <si>
-    <t xml:space="preserve">
-Test plan
-测试计划</t>
+    <t>Test plan</t>
   </si>
   <si>
     <t>Mj50</t>
   </si>
   <si>
-    <t>Test plan
-测试计划</t>
-  </si>
-  <si>
     <t>Master test plan covering normal, alternative and exception paths
-覆盖正常、替代、异常路径的测试计划主文档
 due: Day 1-5</t>
   </si>
   <si>
-    <t>Total
-合计</t>
+    <t>Total</t>
   </si>
   <si>
     <t/>
@@ -328,7 +279,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -367,13 +318,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -518,7 +462,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -557,12 +501,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -730,7 +668,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -751,19 +689,6 @@
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFBFBFBF"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -891,152 +816,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1057,7 +982,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1066,30 +991,11 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1473,382 +1379,380 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:8">
-      <c r="A5" s="5" t="s">
-        <v>3</v>
-      </c>
+      <c r="A5" s="5"/>
     </row>
     <row r="7" ht="61" customHeight="1" spans="1:8">
       <c r="A7" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>10</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1" spans="1:8">
       <c r="A8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="D8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="E8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="F8" s="7" t="s">
         <v>16</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>17</v>
       </c>
       <c r="G8" s="7">
         <v>18</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1" spans="1:8">
       <c r="A9" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="E9" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>21</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>22</v>
       </c>
       <c r="G9" s="10">
         <v>5</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" ht="51" customHeight="1" spans="1:8">
       <c r="A10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>27</v>
-      </c>
       <c r="E10" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G10" s="7">
         <v>8</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" ht="51" customHeight="1" spans="1:8">
       <c r="A11" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="E11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="F11" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G11" s="10">
         <v>5</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" ht="51" customHeight="1" spans="1:8">
       <c r="A12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="9" t="s">
+      <c r="D12" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="9" t="s">
-        <v>36</v>
-      </c>
       <c r="E12" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G12" s="7">
         <v>5</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" ht="66" customHeight="1" spans="1:8">
       <c r="A13" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="C13" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="D13" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="12" t="s">
-        <v>41</v>
-      </c>
       <c r="E13" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G13" s="10">
         <v>10</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" ht="66" customHeight="1" spans="1:8">
       <c r="A14" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="13"/>
+      <c r="C14" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="9" t="s">
+      <c r="D14" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="E14" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G14" s="7">
         <v>16</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" ht="51" customHeight="1" spans="1:8">
       <c r="A15" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="13"/>
+      <c r="C15" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="12" t="s">
+      <c r="D15" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="12" t="s">
-        <v>49</v>
-      </c>
       <c r="E15" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G15" s="10">
         <v>13</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" ht="66" customHeight="1" spans="1:8">
       <c r="A16" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B16" s="13"/>
+      <c r="C16" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B16" s="16"/>
-      <c r="C16" s="9" t="s">
+      <c r="D16" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>53</v>
-      </c>
       <c r="E16" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G16" s="7">
         <v>8</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" ht="66" customHeight="1" spans="1:8">
       <c r="A17" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="12" t="s">
+      <c r="D17" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="12" t="s">
-        <v>57</v>
-      </c>
       <c r="E17" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G17" s="10">
         <v>13</v>
       </c>
       <c r="H17" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" ht="51" customHeight="1" spans="1:8">
       <c r="A18" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="C18" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="D18" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>62</v>
-      </c>
       <c r="E18" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G18" s="7">
         <v>16</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" ht="51" customHeight="1" spans="1:8">
       <c r="A19" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="C19" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="D19" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="12" t="s">
-        <v>67</v>
-      </c>
       <c r="E19" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G19" s="10">
         <v>26</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" ht="66" customHeight="1" spans="1:8">
       <c r="A20" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="C20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>71</v>
-      </c>
       <c r="D20" s="9" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G20" s="7">
         <v>8</v>
       </c>
       <c r="H20" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1" spans="1:8">
+      <c r="A21" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="21" ht="34" customHeight="1" spans="1:8">
-      <c r="A21" s="20" t="s">
+      <c r="D21" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="G21" s="15">
+        <v>151</v>
+      </c>
+      <c r="H21" s="16" t="s">
         <v>74</v>
-      </c>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="E21" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="F21" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="G21" s="20">
-        <v>151</v>
-      </c>
-      <c r="H21" s="21" t="s">
-        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>